<commit_message>
Use real contract terms; add PDF extraction tooling
- Demo: payment schedule from the real contracts (70/20/10 and 90/10)
  with releasable As-Built / initial-handover holdbacks, planning
  invoices paid 100%, AO financial commitment checks and alerts,
  contract terms (guarantee, delay fines, warranty) in admin.
- Templates: contract and AO headers now carry payment schedule,
  guarantee, fines, stamps, financial commitment, planning annex.
- scripts: extract_boq_pdfs.py (BOQ tables from digital PDFs),
  merge_ao_extracts.py (scanned AO letters/addenda -> AO master),
  reconcile_ao_boq.py (match BOQ files to AOs by value).
- docs: contract terms and schema changes in data-dictionary.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/05_العقد_والمقايسة.xlsx
+++ b/templates/05_العقد_والمقايسة.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -754,88 +754,306 @@
       <c r="D9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>تأمين ضمان الأعمال %</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>نسبة الصرف مع المستخلص الشهري % *</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>retention_pct</t>
+          <t>pay_monthly_pct</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>بيتخصم من كل مستخلص ويتفرج عنه بعد الضمان</t>
+          <t>232: 70% — 231: 90%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>خصم ضريبي من المنبع %</t>
+          <t>نسبة محجوزة لحد تسليم خرائط As-Built %</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>tax_pct</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr"/>
+          <t>pay_asbuilt_pct</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>232: 20% — 231: 0</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>دمغة %</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr"/>
+          <t>نسبة محجوزة لحد التسليم الابتدائي %</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>stamp_pct</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr"/>
+          <t>pay_handover_pct</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>232 و 231: 10%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>الدفعة المقدمة %</t>
+          <t>نسبة صرف أعمال التخطيط %</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>advance_pct</t>
+          <t>planning_pay_pct</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>لو فيه دفعة مقدمة بتسترد من المستخلصات</t>
+          <t>التخطيط بيتصرف 100% بعد الانتهاء منه</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>قيمة العقد</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr"/>
+          <t>خطاب الضمان النهائي % من قيمة أمر التكليف</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>final_guarantee_pct</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>بيتقدم مع كل أمر تكليف</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>غرامة التأخير % لكل أسبوع</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>delay_fine_pct_week</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>231: 2% أسبوعياً</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>الحد الأقصى للغرامة %</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>delay_fine_cap_pct</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>من قيمة الأعمال المتأخرة</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>مدة الضمان الفني (شهور)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>warranty_months</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>علاوة خارج النطاق</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>5% / 10% / 15% سيناء</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>out_of_scope_uplift</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>حتى 25% (أو حسب ملحق البرقية)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>دمغة المهن الهندسية % (على أمر التكليف)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>stamp_engineering_pct</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>بتتدفع مرة واحدة مع أمر التكليف</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>دمغة مصممي الفنون التطبيقية %</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>stamp_applied_arts_pct</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>دمغة التشييد والبناء %</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>stamp_construction_pct</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>خصم ضريبي من المنبع %</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>tax_pct</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>من المالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>تأمين ضمان أعمال إضافي % (لو موجود)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>retention_pct</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>العقود الحالية مفيهاش — الضمان بخطاب ضمان نهائي</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>الدفعة المقدمة % (لو موجودة)</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>advance_pct</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>العقود الحالية مفيهاش دفعة مقدمة</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>قيمة العقد (بعد آخر ملحق)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
           <t>contract_value</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>لو فاضي بتتحسب من المقايسة</t>
         </is>

</xml_diff>